<commit_message>
add 2017 local elections
</commit_message>
<xml_diff>
--- a/src/data/raw/local2021_elected_people.xlsx
+++ b/src/data/raw/local2021_elected_people.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox (Personal)\My projects\Elections\ge_elections_dashboard\wireframe\observable_framework\elections_data\src\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA7098A-C9FE-4245-84F3-CB2CEDF3CBEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC969423-AF01-4D79-BCAA-B84798C2B96E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8579,6 +8579,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K2091"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="17.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.3046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="76.07421875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.23046875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A1" t="s">

</xml_diff>